<commit_message>
Rocerd recent progress in Q=const sampling of NGC188
</commit_message>
<xml_diff>
--- a/data/Geller_et_al_2009_WIYN_single_lined_orbits.xlsx
+++ b/data/Geller_et_al_2009_WIYN_single_lined_orbits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpenev/projects/git/CircularizationDissipationConstraints/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B30B43C-4C22-6547-A067-4181393BD126}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C927BCED-A3D8-0F4F-BDA9-383459EECE3D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10880" yWindow="2820" windowWidth="40320" windowHeight="25980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -571,7 +571,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -771,6 +771,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF00F4FF"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -950,7 +956,6 @@
     <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -959,6 +964,7 @@
     <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="16"/>
     <xf numFmtId="0" fontId="20" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -967,8 +973,8 @@
     <xf numFmtId="11" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="22" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1739,7 +1745,7 @@
       <c r="C80" s="1"/>
     </row>
     <row r="81" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A81" s="14" t="s">
+      <c r="A81" s="13" t="s">
         <v>116</v>
       </c>
       <c r="B81" t="s">
@@ -2026,86 +2032,86 @@
         <v>97</v>
       </c>
     </row>
-    <row r="90" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="8" t="s">
+    <row r="90" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="B90" s="8" t="s">
+      <c r="B90" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C90" s="9" t="s">
+      <c r="C90" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D90" s="10">
+      <c r="D90" s="9">
         <v>5362</v>
       </c>
-      <c r="E90" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="F90" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G90" s="11">
+      <c r="E90" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F90" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="G90" s="10">
         <v>6.1894400000000003</v>
       </c>
-      <c r="H90" s="11">
+      <c r="H90" s="10">
         <v>1.9000000000000001E-4</v>
       </c>
-      <c r="I90" s="11">
+      <c r="I90" s="10">
         <v>178.9</v>
       </c>
-      <c r="J90" s="11">
+      <c r="J90" s="10">
         <v>-28.2</v>
       </c>
-      <c r="K90" s="11">
+      <c r="K90" s="10">
         <v>0.3</v>
       </c>
-      <c r="L90" s="11">
+      <c r="L90" s="10">
         <v>49</v>
       </c>
-      <c r="M90" s="11">
+      <c r="M90" s="10">
         <v>0.5</v>
       </c>
-      <c r="N90" s="11">
+      <c r="N90" s="10">
         <v>2.7E-2</v>
       </c>
-      <c r="O90" s="11">
+      <c r="O90" s="10">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="P90" s="11">
+      <c r="P90" s="10">
         <v>183</v>
       </c>
-      <c r="Q90" s="11">
+      <c r="Q90" s="10">
         <v>20</v>
       </c>
-      <c r="R90" s="11">
+      <c r="R90" s="10">
         <v>51035.3</v>
       </c>
-      <c r="S90" s="11">
+      <c r="S90" s="10">
         <v>0.4</v>
       </c>
-      <c r="T90" s="11">
+      <c r="T90" s="10">
         <v>4.17</v>
       </c>
-      <c r="U90" s="11">
+      <c r="U90" s="10">
         <v>0.04</v>
       </c>
-      <c r="V90" s="12">
+      <c r="V90" s="11">
         <v>7.5200000000000003E-2</v>
       </c>
-      <c r="W90" s="12">
+      <c r="W90" s="11">
         <v>2.2000000000000001E-3</v>
       </c>
-      <c r="X90" s="11">
+      <c r="X90" s="10">
         <v>1.51</v>
       </c>
-      <c r="Y90" s="11">
+      <c r="Y90" s="10">
         <v>29</v>
       </c>
-      <c r="Z90" s="11" t="s">
+      <c r="Z90" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="AA90" s="11" t="s">
+      <c r="AA90" s="10" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2269,91 +2275,91 @@
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="8" t="s">
+    <row r="93" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A93" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="B93" s="13" t="s">
+      <c r="B93" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="C93" s="9" t="s">
+      <c r="C93" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D93" s="10">
+      <c r="D93" s="9">
         <v>5733</v>
       </c>
-      <c r="E93" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="F93" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G93" s="11">
+      <c r="E93" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F93" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="G93" s="10">
         <v>8.7040000000000006</v>
       </c>
-      <c r="H93" s="11">
+      <c r="H93" s="10">
         <v>4.0000000000000002E-4</v>
       </c>
-      <c r="I93" s="11">
+      <c r="I93" s="10">
         <v>356.8</v>
       </c>
-      <c r="J93" s="11">
+      <c r="J93" s="10">
         <v>-33</v>
       </c>
-      <c r="K93" s="11">
+      <c r="K93" s="10">
         <v>2.2000000000000002</v>
       </c>
-      <c r="L93" s="11">
+      <c r="L93" s="10">
         <v>60</v>
       </c>
-      <c r="M93" s="11">
+      <c r="M93" s="10">
         <v>5</v>
       </c>
-      <c r="N93" s="11">
+      <c r="N93" s="10">
         <v>0.5</v>
       </c>
-      <c r="O93" s="11">
+      <c r="O93" s="10">
         <v>0.05</v>
       </c>
-      <c r="P93" s="11">
+      <c r="P93" s="10">
         <v>120</v>
       </c>
-      <c r="Q93" s="11">
+      <c r="Q93" s="10">
         <v>7</v>
       </c>
-      <c r="R93" s="11">
+      <c r="R93" s="10">
         <v>51606.69</v>
       </c>
-      <c r="S93" s="11">
+      <c r="S93" s="10">
         <v>0.1</v>
       </c>
-      <c r="T93" s="11">
+      <c r="T93" s="10">
         <v>6.2</v>
       </c>
-      <c r="U93" s="11">
+      <c r="U93" s="10">
         <v>0.6</v>
       </c>
-      <c r="V93" s="12">
+      <c r="V93" s="11">
         <v>0.13</v>
       </c>
-      <c r="W93" s="12">
+      <c r="W93" s="11">
         <v>0.03</v>
       </c>
-      <c r="X93" s="11">
+      <c r="X93" s="10">
         <v>5.49</v>
       </c>
-      <c r="Y93" s="11">
+      <c r="Y93" s="10">
         <v>11</v>
       </c>
-      <c r="Z93" s="11" t="s">
+      <c r="Z93" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="AA93" s="11" t="s">
+      <c r="AA93" s="10" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="94" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A94" s="14" t="s">
+      <c r="A94" s="13" t="s">
         <v>113</v>
       </c>
       <c r="B94" s="5" t="s">
@@ -2436,7 +2442,7 @@
       </c>
     </row>
     <row r="95" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A95" s="14" t="s">
+      <c r="A95" s="13" t="s">
         <v>113</v>
       </c>
       <c r="B95" s="5" t="s">
@@ -2519,7 +2525,7 @@
       </c>
     </row>
     <row r="96" spans="1:27" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="14" t="s">
+      <c r="A96" s="13" t="s">
         <v>113</v>
       </c>
       <c r="B96" s="24" t="s">
@@ -2685,7 +2691,7 @@
       </c>
     </row>
     <row r="98" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A98" s="14" t="s">
+      <c r="A98" s="13" t="s">
         <v>113</v>
       </c>
       <c r="B98" s="5" t="s">
@@ -2768,7 +2774,7 @@
       </c>
     </row>
     <row r="99" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A99" s="14" t="s">
+      <c r="A99" s="13" t="s">
         <v>113</v>
       </c>
       <c r="B99" s="5" t="s">
@@ -2850,91 +2856,91 @@
         <v>97</v>
       </c>
     </row>
-    <row r="100" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="15" t="s">
+    <row r="100" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A100" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="B100" s="13" t="s">
+      <c r="B100" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="C100" s="9" t="s">
+      <c r="C100" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D100" s="10">
+      <c r="D100" s="9">
         <v>8775</v>
       </c>
-      <c r="E100" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="F100" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G100" s="11">
+      <c r="E100" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F100" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="G100" s="10">
         <v>14.57</v>
       </c>
-      <c r="H100" s="11">
+      <c r="H100" s="10">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="I100" s="11">
+      <c r="I100" s="10">
         <v>50.8</v>
       </c>
-      <c r="J100" s="11">
+      <c r="J100" s="10">
         <v>-23.18</v>
       </c>
-      <c r="K100" s="11">
+      <c r="K100" s="10">
         <v>0.22</v>
       </c>
-      <c r="L100" s="11">
+      <c r="L100" s="10">
         <v>8.8000000000000007</v>
       </c>
-      <c r="M100" s="11">
+      <c r="M100" s="10">
         <v>0.3</v>
       </c>
-      <c r="N100" s="11">
+      <c r="N100" s="10">
         <v>0.2</v>
       </c>
-      <c r="O100" s="11">
+      <c r="O100" s="10">
         <v>0.04</v>
       </c>
-      <c r="P100" s="11">
+      <c r="P100" s="10">
         <v>74</v>
       </c>
-      <c r="Q100" s="11">
+      <c r="Q100" s="10">
         <v>9</v>
       </c>
-      <c r="R100" s="11">
+      <c r="R100" s="10">
         <v>50890.400000000001</v>
       </c>
-      <c r="S100" s="11">
+      <c r="S100" s="10">
         <v>0.3</v>
       </c>
-      <c r="T100" s="11">
+      <c r="T100" s="10">
         <v>1.72</v>
       </c>
-      <c r="U100" s="11">
+      <c r="U100" s="10">
         <v>0.06</v>
       </c>
-      <c r="V100" s="12">
+      <c r="V100" s="11">
         <v>9.6000000000000002E-4</v>
       </c>
-      <c r="W100" s="12">
+      <c r="W100" s="11">
         <v>1E-4</v>
       </c>
-      <c r="X100" s="11">
+      <c r="X100" s="10">
         <v>0.9</v>
       </c>
-      <c r="Y100" s="11">
+      <c r="Y100" s="10">
         <v>19</v>
       </c>
-      <c r="Z100" s="11" t="s">
+      <c r="Z100" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="AA100" s="11" t="s">
+      <c r="AA100" s="10" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="101" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A101" s="14" t="s">
+      <c r="A101" s="13" t="s">
         <v>113</v>
       </c>
       <c r="B101" s="5" t="s">
@@ -3017,10 +3023,10 @@
       </c>
     </row>
     <row r="102" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A102" s="14" t="s">
+      <c r="A102" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="B102" s="7" t="s">
+      <c r="B102" s="5" t="s">
         <v>112</v>
       </c>
       <c r="C102" s="1" t="s">
@@ -3100,10 +3106,10 @@
       </c>
     </row>
     <row r="103" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A103" s="14" t="s">
+      <c r="A103" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="B103" s="7" t="s">
+      <c r="B103" s="5" t="s">
         <v>112</v>
       </c>
       <c r="C103" s="1" t="s">
@@ -3183,7 +3189,7 @@
       </c>
     </row>
     <row r="104" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="B104" s="7" t="s">
+      <c r="B104" s="5" t="s">
         <v>112</v>
       </c>
       <c r="C104" s="1" t="s">
@@ -3263,7 +3269,7 @@
       </c>
     </row>
     <row r="105" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="B105" s="7" t="s">
+      <c r="B105" s="5" t="s">
         <v>112</v>
       </c>
       <c r="C105" s="1" t="s">
@@ -3419,157 +3425,157 @@
         <v>97</v>
       </c>
     </row>
-    <row r="107" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C107" s="9" t="s">
+    <row r="107" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="C107" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D107" s="11">
+      <c r="D107" s="10">
         <v>5110</v>
       </c>
-      <c r="E107" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="F107" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G107" s="11">
+      <c r="E107" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F107" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="G107" s="10">
         <v>21.360199999999999</v>
       </c>
-      <c r="H107" s="11">
+      <c r="H107" s="10">
         <v>1.9E-3</v>
       </c>
-      <c r="I107" s="11">
+      <c r="I107" s="10">
         <v>163.19999999999999</v>
       </c>
-      <c r="J107" s="11">
+      <c r="J107" s="10">
         <v>-38</v>
       </c>
-      <c r="K107" s="11">
+      <c r="K107" s="10">
         <v>0.7</v>
       </c>
-      <c r="L107" s="11">
+      <c r="L107" s="10">
         <v>37.799999999999997</v>
       </c>
-      <c r="M107" s="11">
+      <c r="M107" s="10">
         <v>0.9</v>
       </c>
-      <c r="N107" s="11">
+      <c r="N107" s="10">
         <v>0.1</v>
       </c>
-      <c r="O107" s="11">
+      <c r="O107" s="10">
         <v>0.03</v>
       </c>
-      <c r="P107" s="11">
+      <c r="P107" s="10">
         <v>195</v>
       </c>
-      <c r="Q107" s="11">
+      <c r="Q107" s="10">
         <v>16</v>
       </c>
-      <c r="R107" s="11">
+      <c r="R107" s="10">
         <v>51197.2</v>
       </c>
-      <c r="S107" s="11">
+      <c r="S107" s="10">
         <v>0.9</v>
       </c>
-      <c r="T107" s="11">
+      <c r="T107" s="10">
         <v>11.1</v>
       </c>
-      <c r="U107" s="11">
+      <c r="U107" s="10">
         <v>0.3</v>
       </c>
-      <c r="V107" s="12">
+      <c r="V107" s="11">
         <v>0.11799999999999999</v>
       </c>
-      <c r="W107" s="12">
+      <c r="W107" s="11">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="X107" s="11">
+      <c r="X107" s="10">
         <v>3.07</v>
       </c>
-      <c r="Y107" s="11">
+      <c r="Y107" s="10">
         <v>22</v>
       </c>
-      <c r="Z107" s="11" t="s">
+      <c r="Z107" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="AA107" s="11" t="s">
+      <c r="AA107" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="108" spans="1:27" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C108" s="9" t="s">
+    <row r="108" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="C108" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D108" s="11">
+      <c r="D108" s="10">
         <v>736</v>
       </c>
-      <c r="E108" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="F108" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G108" s="11">
+      <c r="E108" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F108" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="G108" s="10">
         <v>24.004000000000001</v>
       </c>
-      <c r="H108" s="11">
+      <c r="H108" s="10">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="I108" s="11">
+      <c r="I108" s="10">
         <v>50.8</v>
       </c>
-      <c r="J108" s="11">
+      <c r="J108" s="10">
         <v>-50.5</v>
       </c>
-      <c r="K108" s="11">
+      <c r="K108" s="10">
         <v>0.11</v>
       </c>
-      <c r="L108" s="11">
+      <c r="L108" s="10">
         <v>7.21</v>
       </c>
-      <c r="M108" s="11">
+      <c r="M108" s="10">
         <v>0.16</v>
       </c>
-      <c r="N108" s="11">
+      <c r="N108" s="10">
         <v>0.21</v>
       </c>
-      <c r="O108" s="11">
+      <c r="O108" s="10">
         <v>1.9E-2</v>
       </c>
-      <c r="P108" s="11">
+      <c r="P108" s="10">
         <v>240</v>
       </c>
-      <c r="Q108" s="11">
+      <c r="Q108" s="10">
         <v>6</v>
       </c>
-      <c r="R108" s="11">
+      <c r="R108" s="10">
         <v>52039.8</v>
       </c>
-      <c r="S108" s="11">
+      <c r="S108" s="10">
         <v>0.4</v>
       </c>
-      <c r="T108" s="11">
+      <c r="T108" s="10">
         <v>2.33</v>
       </c>
-      <c r="U108" s="11">
+      <c r="U108" s="10">
         <v>0.05</v>
       </c>
-      <c r="V108" s="12">
+      <c r="V108" s="11">
         <v>8.7000000000000001E-4</v>
       </c>
-      <c r="W108" s="12">
+      <c r="W108" s="11">
         <v>6.0000000000000002E-5</v>
       </c>
-      <c r="X108" s="11">
+      <c r="X108" s="10">
         <v>0.42</v>
       </c>
-      <c r="Y108" s="11">
+      <c r="Y108" s="10">
         <v>17</v>
       </c>
-      <c r="Z108" s="11" t="s">
+      <c r="Z108" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="AA108" s="11" t="s">
+      <c r="AA108" s="10" t="s">
         <v>97</v>
       </c>
     </row>
@@ -3654,7 +3660,7 @@
       </c>
     </row>
     <row r="110" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="B110" s="25" t="s">
+      <c r="B110" s="15" t="s">
         <v>112</v>
       </c>
       <c r="C110" s="1" t="s">

</xml_diff>

<commit_message>
Mark more sampling progress
</commit_message>
<xml_diff>
--- a/data/Geller_et_al_2009_WIYN_single_lined_orbits.xlsx
+++ b/data/Geller_et_al_2009_WIYN_single_lined_orbits.xlsx
@@ -1,26 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10411"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpenev/projects/git/CircularizationDissipationConstraints/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E090225-8288-5A46-AEC1-CF1F46CC1FFD}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6393DE1-283D-9E4D-B699-BEF321ADA1C4}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10880" yWindow="2820" windowWidth="40320" windowHeight="25980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Geller_et_al_2009_WIYN_single_l" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="128">
   <si>
     <t>#</t>
   </si>
@@ -410,7 +421,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -570,6 +581,14 @@
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF00F4FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -975,7 +994,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -997,11 +1016,14 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="11" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="23" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1799,7 +1821,7 @@
       <c r="C83" s="1"/>
     </row>
     <row r="84" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A84" s="23" t="s">
+      <c r="A84" s="24" t="s">
         <v>116</v>
       </c>
       <c r="B84" t="s">
@@ -1808,7 +1830,7 @@
       <c r="C84" s="1"/>
     </row>
     <row r="85" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A85" s="18" t="s">
+      <c r="A85" s="21" t="s">
         <v>123</v>
       </c>
       <c r="B85" t="s">
@@ -1817,7 +1839,7 @@
       <c r="C85" s="1"/>
     </row>
     <row r="86" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A86" s="25" t="s">
+      <c r="A86" s="26" t="s">
         <v>126</v>
       </c>
       <c r="B86" t="s">
@@ -2155,7 +2177,7 @@
       <c r="A92" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B92" s="5" t="s">
+      <c r="B92" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C92" s="1" t="s">
@@ -2235,6 +2257,12 @@
       </c>
     </row>
     <row r="93" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A93" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B93" s="5" t="s">
+        <v>112</v>
+      </c>
       <c r="C93" s="1" t="s">
         <v>104</v>
       </c>
@@ -2312,10 +2340,10 @@
       </c>
     </row>
     <row r="94" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="5" t="s">
+      <c r="A94" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="B94" s="12" t="s">
+      <c r="B94" s="27" t="s">
         <v>112</v>
       </c>
       <c r="C94" s="8" t="s">
@@ -2395,10 +2423,10 @@
       </c>
     </row>
     <row r="95" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A95" s="16" t="s">
+      <c r="A95" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B95" s="5" t="s">
+      <c r="B95" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C95" s="1" t="s">
@@ -2481,7 +2509,7 @@
       <c r="A96" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B96" s="5" t="s">
+      <c r="B96" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C96" s="1" t="s">
@@ -2561,10 +2589,10 @@
       </c>
     </row>
     <row r="97" spans="1:27" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="16" t="s">
+      <c r="A97" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B97" s="23" t="s">
+      <c r="B97" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C97" s="1" t="s">
@@ -2644,10 +2672,10 @@
       </c>
     </row>
     <row r="98" spans="1:27" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="21" t="s">
+      <c r="A98" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="B98" s="22" t="s">
+      <c r="B98" s="28" t="s">
         <v>112</v>
       </c>
       <c r="C98" s="19" t="s">
@@ -2727,10 +2755,10 @@
       </c>
     </row>
     <row r="99" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A99" s="16" t="s">
+      <c r="A99" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B99" s="5" t="s">
+      <c r="B99" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C99" s="1" t="s">
@@ -2810,10 +2838,10 @@
       </c>
     </row>
     <row r="100" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A100" s="16" t="s">
+      <c r="A100" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B100" s="5" t="s">
+      <c r="B100" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C100" s="1" t="s">
@@ -2979,7 +3007,7 @@
       <c r="A102" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B102" s="5" t="s">
+      <c r="B102" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C102" s="1" t="s">
@@ -3305,7 +3333,7 @@
       </c>
     </row>
     <row r="106" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="B106" s="5" t="s">
+      <c r="B106" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C106" s="1" t="s">
@@ -3384,80 +3412,80 @@
         <v>97</v>
       </c>
     </row>
-    <row r="107" spans="1:27" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C107" s="19" t="s">
+    <row r="107" spans="1:27" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="C107" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="D107" s="18">
+      <c r="D107" s="21">
         <v>4710</v>
       </c>
-      <c r="E107" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="F107" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G107" s="18">
+      <c r="E107" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F107" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="G107" s="21">
         <v>21.340699999999998</v>
       </c>
-      <c r="H107" s="18">
+      <c r="H107" s="21">
         <v>6.9999999999999999E-4</v>
       </c>
-      <c r="I107" s="18">
+      <c r="I107" s="21">
         <v>203.7</v>
       </c>
-      <c r="J107" s="18">
+      <c r="J107" s="21">
         <v>-45.7</v>
       </c>
-      <c r="K107" s="18">
+      <c r="K107" s="21">
         <v>0.3</v>
       </c>
-      <c r="L107" s="18">
+      <c r="L107" s="21">
         <v>16.899999999999999</v>
       </c>
-      <c r="M107" s="18">
+      <c r="M107" s="21">
         <v>1.5</v>
       </c>
-      <c r="N107" s="18">
+      <c r="N107" s="21">
         <v>0.67500000000000004</v>
       </c>
-      <c r="O107" s="18">
+      <c r="O107" s="21">
         <v>2.4E-2</v>
       </c>
-      <c r="P107" s="18">
+      <c r="P107" s="21">
         <v>340</v>
       </c>
-      <c r="Q107" s="18">
+      <c r="Q107" s="21">
         <v>3</v>
       </c>
-      <c r="R107" s="18">
+      <c r="R107" s="21">
         <v>52412.34</v>
       </c>
-      <c r="S107" s="18">
+      <c r="S107" s="21">
         <v>0.16</v>
       </c>
-      <c r="T107" s="18">
+      <c r="T107" s="21">
         <v>3.7</v>
       </c>
-      <c r="U107" s="18">
+      <c r="U107" s="21">
         <v>0.3</v>
       </c>
-      <c r="V107" s="20">
+      <c r="V107" s="23">
         <v>4.3E-3</v>
       </c>
-      <c r="W107" s="20">
+      <c r="W107" s="23">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="X107" s="18">
+      <c r="X107" s="21">
         <v>1.18</v>
       </c>
-      <c r="Y107" s="18">
+      <c r="Y107" s="21">
         <v>37</v>
       </c>
-      <c r="Z107" s="18" t="s">
+      <c r="Z107" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="AA107" s="18" t="s">
+      <c r="AA107" s="21" t="s">
         <v>97</v>
       </c>
     </row>
@@ -3616,7 +3644,7 @@
       </c>
     </row>
     <row r="110" spans="1:27" ht="29" x14ac:dyDescent="0.35">
-      <c r="B110" s="24" t="s">
+      <c r="B110" s="25" t="s">
         <v>125</v>
       </c>
       <c r="C110" s="1" t="s">
@@ -3855,80 +3883,80 @@
         <v>97</v>
       </c>
     </row>
-    <row r="113" spans="3:27" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C113" s="19" t="s">
+    <row r="113" spans="3:27" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="C113" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="D113" s="18">
+      <c r="D113" s="21">
         <v>4673</v>
       </c>
-      <c r="E113" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="F113" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G113" s="18">
+      <c r="E113" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F113" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="G113" s="21">
         <v>48.27</v>
       </c>
-      <c r="H113" s="18">
+      <c r="H113" s="21">
         <v>0.06</v>
       </c>
-      <c r="I113" s="18">
+      <c r="I113" s="21">
         <v>22.4</v>
       </c>
-      <c r="J113" s="18">
+      <c r="J113" s="21">
         <v>-41.35</v>
       </c>
-      <c r="K113" s="18">
+      <c r="K113" s="21">
         <v>0.12</v>
       </c>
-      <c r="L113" s="18">
+      <c r="L113" s="21">
         <v>8.4</v>
       </c>
-      <c r="M113" s="18">
+      <c r="M113" s="21">
         <v>0.3</v>
       </c>
-      <c r="N113" s="18">
+      <c r="N113" s="21">
         <v>0.37</v>
       </c>
-      <c r="O113" s="18">
+      <c r="O113" s="21">
         <v>0.03</v>
       </c>
-      <c r="P113" s="18">
+      <c r="P113" s="21">
         <v>351</v>
       </c>
-      <c r="Q113" s="18">
+      <c r="Q113" s="21">
         <v>4</v>
       </c>
-      <c r="R113" s="18">
+      <c r="R113" s="21">
         <v>50836.6</v>
       </c>
-      <c r="S113" s="18">
+      <c r="S113" s="21">
         <v>0.6</v>
       </c>
-      <c r="T113" s="18">
+      <c r="T113" s="21">
         <v>5.18</v>
       </c>
-      <c r="U113" s="18">
+      <c r="U113" s="21">
         <v>0.19</v>
       </c>
-      <c r="V113" s="20">
+      <c r="V113" s="23">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="W113" s="20">
+      <c r="W113" s="23">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="X113" s="18">
+      <c r="X113" s="21">
         <v>0.49</v>
       </c>
-      <c r="Y113" s="18">
+      <c r="Y113" s="21">
         <v>22</v>
       </c>
-      <c r="Z113" s="18" t="s">
+      <c r="Z113" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="AA113" s="18" t="s">
+      <c r="AA113" s="21" t="s">
         <v>97</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark sampling progress from before discovering issue with e prior
</commit_message>
<xml_diff>
--- a/data/Geller_et_al_2009_WIYN_single_lined_orbits.xlsx
+++ b/data/Geller_et_al_2009_WIYN_single_lined_orbits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpenev/projects/git/CircularizationDissipationConstraints/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6393DE1-283D-9E4D-B699-BEF321ADA1C4}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F21921BA-D6F0-F94E-98E2-FC18C7E7CBB9}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10880" yWindow="2820" windowWidth="40320" windowHeight="25980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2091,7 +2091,7 @@
       </c>
     </row>
     <row r="91" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="7" t="s">
+      <c r="A91" s="5" t="s">
         <v>113</v>
       </c>
       <c r="B91" s="7" t="s">
@@ -2174,7 +2174,7 @@
       </c>
     </row>
     <row r="92" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A92" s="5" t="s">
+      <c r="A92" s="24" t="s">
         <v>113</v>
       </c>
       <c r="B92" s="24" t="s">
@@ -2340,7 +2340,7 @@
       </c>
     </row>
     <row r="94" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="12" t="s">
+      <c r="A94" s="27" t="s">
         <v>113</v>
       </c>
       <c r="B94" s="27" t="s">
@@ -2838,7 +2838,7 @@
       </c>
     </row>
     <row r="100" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A100" s="5" t="s">
+      <c r="A100" s="24" t="s">
         <v>113</v>
       </c>
       <c r="B100" s="24" t="s">
@@ -2921,7 +2921,7 @@
       </c>
     </row>
     <row r="101" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="5" t="s">
+      <c r="A101" s="27" t="s">
         <v>113</v>
       </c>
       <c r="B101" s="12" t="s">
@@ -3173,7 +3173,7 @@
       <c r="A104" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B104" s="5" t="s">
+      <c r="B104" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C104" s="1" t="s">
@@ -3724,7 +3724,7 @@
       </c>
     </row>
     <row r="111" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="B111" s="14" t="s">
+      <c r="B111" s="24" t="s">
         <v>112</v>
       </c>
       <c r="C111" s="1" t="s">

</xml_diff>

<commit_message>
Record progress after first complete round of sampling
</commit_message>
<xml_diff>
--- a/data/Geller_et_al_2009_WIYN_single_lined_orbits.xlsx
+++ b/data/Geller_et_al_2009_WIYN_single_lined_orbits.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10411"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpenev/projects/git/CircularizationDissipationConstraints/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F21921BA-D6F0-F94E-98E2-FC18C7E7CBB9}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA1DA070-F668-1B46-883E-CA921A991C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10880" yWindow="2820" windowWidth="40320" windowHeight="25980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="500" windowWidth="33600" windowHeight="20540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Geller_et_al_2009_WIYN_single_l" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="126">
   <si>
     <t>#</t>
   </si>
@@ -363,21 +363,12 @@
     <t>Units</t>
   </si>
   <si>
-    <t>Q=const</t>
-  </si>
-  <si>
     <t>Q=pwrlaw</t>
   </si>
   <si>
-    <t>ganymede</t>
-  </si>
-  <si>
     <t>stampede</t>
   </si>
   <si>
-    <t>kartof</t>
-  </si>
-  <si>
     <t>Color codes</t>
   </si>
   <si>
@@ -408,13 +399,16 @@
     <t>Sufficient samples accumulated on the given cluster</t>
   </si>
   <si>
-    <t>CRASHED</t>
-  </si>
-  <si>
     <t>bold purple</t>
   </si>
   <si>
     <t>Stellar mass distributions go out of range too often</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>M but PPM/PRV small</t>
   </si>
 </sst>
 </file>
@@ -585,14 +579,6 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="FF00F4FF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
       <color rgb="FF00C8D2"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -616,8 +602,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="39">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -817,19 +809,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF00F4FF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -994,7 +974,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1002,28 +982,27 @@
     <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="16"/>
     <xf numFmtId="0" fontId="20" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="11" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="11" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="24" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1073,8 +1052,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF00C8D2"/>
       <color rgb="FF00F4FF"/>
-      <color rgb="FF00C8D2"/>
       <color rgb="FF009EFF"/>
       <color rgb="FFFF7D41"/>
       <color rgb="FF009099"/>
@@ -1395,6 +1374,7 @@
   <cols>
     <col min="1" max="1" width="15.1640625" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:3" x14ac:dyDescent="0.2">
@@ -1788,71 +1768,71 @@
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A80" s="15" t="s">
+      <c r="A80" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="C80" s="1"/>
+    </row>
+    <row r="81" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A81" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="B81" t="s">
+        <v>114</v>
+      </c>
+      <c r="C81" s="1"/>
+    </row>
+    <row r="82" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A82" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="B82" t="s">
         <v>115</v>
-      </c>
-      <c r="C80" s="1"/>
-    </row>
-    <row r="81" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A81" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="B81" t="s">
-        <v>117</v>
-      </c>
-      <c r="C81" s="1"/>
-    </row>
-    <row r="82" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A82" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="B82" t="s">
-        <v>118</v>
       </c>
       <c r="C82" s="1"/>
     </row>
     <row r="83" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A83" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B83" t="s">
         <v>116</v>
       </c>
-      <c r="B83" t="s">
+      <c r="C83" s="1"/>
+    </row>
+    <row r="84" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A84" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84" t="s">
+        <v>121</v>
+      </c>
+      <c r="C84" s="1"/>
+    </row>
+    <row r="85" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A85" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B85" t="s">
         <v>119</v>
       </c>
-      <c r="C83" s="1"/>
-    </row>
-    <row r="84" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A84" s="24" t="s">
-        <v>116</v>
-      </c>
-      <c r="B84" t="s">
-        <v>124</v>
-      </c>
-      <c r="C84" s="1"/>
-    </row>
-    <row r="85" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A85" s="21" t="s">
+      <c r="C85" s="1"/>
+    </row>
+    <row r="86" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A86" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="B86" t="s">
         <v>123</v>
       </c>
-      <c r="B85" t="s">
-        <v>122</v>
-      </c>
-      <c r="C85" s="1"/>
-    </row>
-    <row r="86" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A86" s="26" t="s">
-        <v>126</v>
-      </c>
-      <c r="B86" t="s">
-        <v>127</v>
-      </c>
       <c r="C86" s="1"/>
     </row>
     <row r="87" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A87" s="17" t="s">
-        <v>121</v>
+      <c r="A87" s="14" t="s">
+        <v>118</v>
       </c>
       <c r="B87" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C87" s="1"/>
     </row>
@@ -1890,7 +1870,7 @@
       <c r="M88" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="N88" s="3" t="s">
+      <c r="N88" s="20" t="s">
         <v>98</v>
       </c>
       <c r="O88" s="3" t="s">
@@ -1932,10 +1912,10 @@
     </row>
     <row r="89" spans="1:27" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>73</v>
@@ -1970,7 +1950,7 @@
       <c r="M89" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="N89" s="3" t="s">
+      <c r="N89" s="20" t="s">
         <v>84</v>
       </c>
       <c r="O89" s="3" t="s">
@@ -2014,6 +1994,9 @@
       </c>
     </row>
     <row r="90" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A90" s="13" t="s">
+        <v>111</v>
+      </c>
       <c r="C90" s="1" t="s">
         <v>104</v>
       </c>
@@ -2047,7 +2030,7 @@
       <c r="M90">
         <v>0.3</v>
       </c>
-      <c r="N90">
+      <c r="N90" s="5">
         <v>0.05</v>
       </c>
       <c r="O90">
@@ -2090,96 +2073,90 @@
         <v>97</v>
       </c>
     </row>
-    <row r="91" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B91" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C91" s="8" t="s">
+    <row r="91" spans="1:27" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="6"/>
+      <c r="B91" s="8"/>
+      <c r="C91" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D91" s="9">
+      <c r="D91" s="8">
         <v>5362</v>
       </c>
-      <c r="E91" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="F91" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="G91" s="10">
+      <c r="E91" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F91" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G91" s="9">
         <v>6.1894400000000003</v>
       </c>
-      <c r="H91" s="10">
+      <c r="H91" s="9">
         <v>1.9000000000000001E-4</v>
       </c>
-      <c r="I91" s="10">
+      <c r="I91" s="9">
         <v>178.9</v>
       </c>
-      <c r="J91" s="10">
+      <c r="J91" s="9">
         <v>-28.2</v>
       </c>
-      <c r="K91" s="10">
+      <c r="K91" s="9">
         <v>0.3</v>
       </c>
-      <c r="L91" s="10">
+      <c r="L91" s="9">
         <v>49</v>
       </c>
-      <c r="M91" s="10">
+      <c r="M91" s="9">
         <v>0.5</v>
       </c>
-      <c r="N91" s="10">
+      <c r="N91" s="21">
         <v>2.7E-2</v>
       </c>
-      <c r="O91" s="10">
+      <c r="O91" s="9">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="P91" s="10">
+      <c r="P91" s="9">
         <v>183</v>
       </c>
-      <c r="Q91" s="10">
+      <c r="Q91" s="9">
         <v>20</v>
       </c>
-      <c r="R91" s="10">
+      <c r="R91" s="9">
         <v>51035.3</v>
       </c>
-      <c r="S91" s="10">
+      <c r="S91" s="9">
         <v>0.4</v>
       </c>
-      <c r="T91" s="10">
+      <c r="T91" s="9">
         <v>4.17</v>
       </c>
-      <c r="U91" s="10">
+      <c r="U91" s="9">
         <v>0.04</v>
       </c>
-      <c r="V91" s="11">
+      <c r="V91" s="10">
         <v>7.5200000000000003E-2</v>
       </c>
-      <c r="W91" s="11">
+      <c r="W91" s="10">
         <v>2.2000000000000001E-3</v>
       </c>
-      <c r="X91" s="10">
+      <c r="X91" s="9">
         <v>1.51</v>
       </c>
-      <c r="Y91" s="10">
+      <c r="Y91" s="9">
         <v>29</v>
       </c>
-      <c r="Z91" s="10" t="s">
+      <c r="Z91" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="AA91" s="10" t="s">
+      <c r="AA91" s="9" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="92" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A92" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="B92" s="24" t="s">
-        <v>112</v>
-      </c>
+      <c r="A92" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B92" s="6"/>
       <c r="C92" s="1" t="s">
         <v>104</v>
       </c>
@@ -2213,7 +2190,7 @@
       <c r="M92">
         <v>0.4</v>
       </c>
-      <c r="N92">
+      <c r="N92" s="5">
         <v>1.7000000000000001E-2</v>
       </c>
       <c r="O92">
@@ -2257,12 +2234,10 @@
       </c>
     </row>
     <row r="93" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A93" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="B93" s="5" t="s">
-        <v>112</v>
-      </c>
+      <c r="A93" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B93" s="6"/>
       <c r="C93" s="1" t="s">
         <v>104</v>
       </c>
@@ -2296,7 +2271,7 @@
       <c r="M93">
         <v>0.7</v>
       </c>
-      <c r="N93">
+      <c r="N93" s="5">
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="O93">
@@ -2339,96 +2314,90 @@
         <v>97</v>
       </c>
     </row>
-    <row r="94" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="B94" s="27" t="s">
-        <v>112</v>
-      </c>
-      <c r="C94" s="8" t="s">
+    <row r="94" spans="1:27" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A94" s="8"/>
+      <c r="B94" s="8"/>
+      <c r="C94" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D94" s="9">
+      <c r="D94" s="8">
         <v>5733</v>
       </c>
-      <c r="E94" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="F94" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="G94" s="10">
+      <c r="E94" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F94" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G94" s="9">
         <v>8.7040000000000006</v>
       </c>
-      <c r="H94" s="10">
+      <c r="H94" s="9">
         <v>4.0000000000000002E-4</v>
       </c>
-      <c r="I94" s="10">
+      <c r="I94" s="9">
         <v>356.8</v>
       </c>
-      <c r="J94" s="10">
+      <c r="J94" s="9">
         <v>-33</v>
       </c>
-      <c r="K94" s="10">
+      <c r="K94" s="9">
         <v>2.2000000000000002</v>
       </c>
-      <c r="L94" s="10">
+      <c r="L94" s="9">
         <v>60</v>
       </c>
-      <c r="M94" s="10">
+      <c r="M94" s="9">
         <v>5</v>
       </c>
-      <c r="N94" s="10">
+      <c r="N94" s="21">
         <v>0.5</v>
       </c>
-      <c r="O94" s="10">
+      <c r="O94" s="9">
         <v>0.05</v>
       </c>
-      <c r="P94" s="10">
+      <c r="P94" s="9">
         <v>120</v>
       </c>
-      <c r="Q94" s="10">
+      <c r="Q94" s="9">
         <v>7</v>
       </c>
-      <c r="R94" s="10">
+      <c r="R94" s="9">
         <v>51606.69</v>
       </c>
-      <c r="S94" s="10">
+      <c r="S94" s="9">
         <v>0.1</v>
       </c>
-      <c r="T94" s="10">
+      <c r="T94" s="9">
         <v>6.2</v>
       </c>
-      <c r="U94" s="10">
+      <c r="U94" s="9">
         <v>0.6</v>
       </c>
-      <c r="V94" s="11">
+      <c r="V94" s="10">
         <v>0.13</v>
       </c>
-      <c r="W94" s="11">
+      <c r="W94" s="10">
         <v>0.03</v>
       </c>
-      <c r="X94" s="10">
+      <c r="X94" s="9">
         <v>5.49</v>
       </c>
-      <c r="Y94" s="10">
+      <c r="Y94" s="9">
         <v>11</v>
       </c>
-      <c r="Z94" s="10" t="s">
+      <c r="Z94" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="AA94" s="10" t="s">
+      <c r="AA94" s="9" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="95" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A95" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B95" s="24" t="s">
-        <v>112</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="B95" s="6"/>
       <c r="C95" s="1" t="s">
         <v>104</v>
       </c>
@@ -2462,7 +2431,7 @@
       <c r="M95">
         <v>0.4</v>
       </c>
-      <c r="N95">
+      <c r="N95" s="5">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="O95">
@@ -2506,12 +2475,10 @@
       </c>
     </row>
     <row r="96" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A96" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B96" s="24" t="s">
-        <v>112</v>
-      </c>
+      <c r="A96" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B96" s="6"/>
       <c r="C96" s="1" t="s">
         <v>104</v>
       </c>
@@ -2545,7 +2512,7 @@
       <c r="M96">
         <v>0.22</v>
       </c>
-      <c r="N96">
+      <c r="N96" s="5">
         <v>0.05</v>
       </c>
       <c r="O96">
@@ -2590,11 +2557,9 @@
     </row>
     <row r="97" spans="1:27" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B97" s="24" t="s">
-        <v>112</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="B97" s="6"/>
       <c r="C97" s="1" t="s">
         <v>104</v>
       </c>
@@ -2628,7 +2593,7 @@
       <c r="M97">
         <v>0.1</v>
       </c>
-      <c r="N97">
+      <c r="N97" s="5">
         <v>0.09</v>
       </c>
       <c r="O97">
@@ -2671,96 +2636,91 @@
         <v>97</v>
       </c>
     </row>
-    <row r="98" spans="1:27" s="18" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="28" t="s">
-        <v>114</v>
-      </c>
-      <c r="B98" s="28" t="s">
-        <v>112</v>
-      </c>
-      <c r="C98" s="19" t="s">
+    <row r="98" spans="1:27" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A98" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C98" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="D98" s="18">
+      <c r="D98" s="23">
         <v>4904</v>
       </c>
-      <c r="E98" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="F98" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="G98" s="18">
+      <c r="E98" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="F98" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="G98" s="23">
         <v>10.185</v>
       </c>
-      <c r="H98" s="18">
+      <c r="H98" s="23">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="I98" s="18">
+      <c r="I98" s="23">
         <v>100.5</v>
       </c>
-      <c r="J98" s="18">
+      <c r="J98" s="23">
         <v>-42.7</v>
       </c>
-      <c r="K98" s="18">
+      <c r="K98" s="23">
         <v>0.3</v>
       </c>
-      <c r="L98" s="18">
+      <c r="L98" s="23">
         <v>11.2</v>
       </c>
-      <c r="M98" s="18">
+      <c r="M98" s="23">
         <v>0.5</v>
       </c>
-      <c r="N98" s="18">
+      <c r="N98" s="25">
         <v>0.37</v>
       </c>
-      <c r="O98" s="18">
+      <c r="O98" s="23">
         <v>0.04</v>
       </c>
-      <c r="P98" s="18">
+      <c r="P98" s="23">
         <v>253</v>
       </c>
-      <c r="Q98" s="18">
+      <c r="Q98" s="23">
         <v>7</v>
       </c>
-      <c r="R98" s="18">
+      <c r="R98" s="23">
         <v>50894.6</v>
       </c>
-      <c r="S98" s="18">
+      <c r="S98" s="23">
         <v>0.16</v>
       </c>
-      <c r="T98" s="18">
+      <c r="T98" s="23">
         <v>1.45</v>
       </c>
-      <c r="U98" s="18">
+      <c r="U98" s="23">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="V98" s="20">
+      <c r="V98" s="26">
         <v>1.1800000000000001E-3</v>
       </c>
-      <c r="W98" s="20">
+      <c r="W98" s="26">
         <v>1.6000000000000001E-4</v>
       </c>
-      <c r="X98" s="18">
+      <c r="X98" s="23">
         <v>1.26</v>
       </c>
-      <c r="Y98" s="18">
+      <c r="Y98" s="23">
         <v>28</v>
       </c>
-      <c r="Z98" s="18" t="s">
+      <c r="Z98" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="AA98" s="18" t="s">
+      <c r="AA98" s="23" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="99" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A99" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B99" s="24" t="s">
-        <v>112</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="B99" s="6"/>
       <c r="C99" s="1" t="s">
         <v>104</v>
       </c>
@@ -2794,7 +2754,7 @@
       <c r="M99">
         <v>0.3</v>
       </c>
-      <c r="N99">
+      <c r="N99" s="5">
         <v>1.2E-2</v>
       </c>
       <c r="O99">
@@ -2838,12 +2798,10 @@
       </c>
     </row>
     <row r="100" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A100" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="B100" s="24" t="s">
-        <v>112</v>
-      </c>
+      <c r="A100" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B100" s="6"/>
       <c r="C100" s="1" t="s">
         <v>104</v>
       </c>
@@ -2877,7 +2835,7 @@
       <c r="M100">
         <v>0.2</v>
       </c>
-      <c r="N100">
+      <c r="N100" s="5">
         <v>0.02</v>
       </c>
       <c r="O100">
@@ -2920,96 +2878,90 @@
         <v>97</v>
       </c>
     </row>
-    <row r="101" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="B101" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C101" s="8" t="s">
+    <row r="101" spans="1:27" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A101" s="8"/>
+      <c r="B101" s="8"/>
+      <c r="C101" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D101" s="9">
+      <c r="D101" s="8">
         <v>8775</v>
       </c>
-      <c r="E101" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="F101" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="G101" s="10">
+      <c r="E101" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F101" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G101" s="9">
         <v>14.57</v>
       </c>
-      <c r="H101" s="10">
+      <c r="H101" s="9">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="I101" s="10">
+      <c r="I101" s="9">
         <v>50.8</v>
       </c>
-      <c r="J101" s="10">
+      <c r="J101" s="9">
         <v>-23.18</v>
       </c>
-      <c r="K101" s="10">
+      <c r="K101" s="9">
         <v>0.22</v>
       </c>
-      <c r="L101" s="10">
+      <c r="L101" s="9">
         <v>8.8000000000000007</v>
       </c>
-      <c r="M101" s="10">
+      <c r="M101" s="9">
         <v>0.3</v>
       </c>
-      <c r="N101" s="10">
+      <c r="N101" s="21">
         <v>0.2</v>
       </c>
-      <c r="O101" s="10">
+      <c r="O101" s="9">
         <v>0.04</v>
       </c>
-      <c r="P101" s="10">
+      <c r="P101" s="9">
         <v>74</v>
       </c>
-      <c r="Q101" s="10">
+      <c r="Q101" s="9">
         <v>9</v>
       </c>
-      <c r="R101" s="10">
+      <c r="R101" s="9">
         <v>50890.400000000001</v>
       </c>
-      <c r="S101" s="10">
+      <c r="S101" s="9">
         <v>0.3</v>
       </c>
-      <c r="T101" s="10">
+      <c r="T101" s="9">
         <v>1.72</v>
       </c>
-      <c r="U101" s="10">
+      <c r="U101" s="9">
         <v>0.06</v>
       </c>
-      <c r="V101" s="11">
+      <c r="V101" s="10">
         <v>9.6000000000000002E-4</v>
       </c>
-      <c r="W101" s="11">
+      <c r="W101" s="10">
         <v>1E-4</v>
       </c>
-      <c r="X101" s="10">
+      <c r="X101" s="9">
         <v>0.9</v>
       </c>
-      <c r="Y101" s="10">
+      <c r="Y101" s="9">
         <v>19</v>
       </c>
-      <c r="Z101" s="10" t="s">
+      <c r="Z101" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="AA101" s="10" t="s">
+      <c r="AA101" s="9" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="102" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A102" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B102" s="24" t="s">
-        <v>112</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="B102" s="6"/>
       <c r="C102" s="1" t="s">
         <v>104</v>
       </c>
@@ -3043,7 +2995,7 @@
       <c r="M102">
         <v>0.19</v>
       </c>
-      <c r="N102">
+      <c r="N102" s="5">
         <v>1.2E-2</v>
       </c>
       <c r="O102">
@@ -3088,11 +3040,9 @@
     </row>
     <row r="103" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A103" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B103" s="5" t="s">
-        <v>112</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="B103" s="6"/>
       <c r="C103" s="1" t="s">
         <v>104</v>
       </c>
@@ -3126,7 +3076,7 @@
       <c r="M103">
         <v>0.2</v>
       </c>
-      <c r="N103">
+      <c r="N103" s="5">
         <v>0.01</v>
       </c>
       <c r="O103">
@@ -3171,11 +3121,9 @@
     </row>
     <row r="104" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A104" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B104" s="24" t="s">
-        <v>112</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="B104" s="6"/>
       <c r="C104" s="1" t="s">
         <v>104</v>
       </c>
@@ -3209,7 +3157,7 @@
       <c r="M104">
         <v>0.23</v>
       </c>
-      <c r="N104">
+      <c r="N104" s="5">
         <v>2.3E-2</v>
       </c>
       <c r="O104">
@@ -3253,9 +3201,10 @@
       </c>
     </row>
     <row r="105" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="B105" s="5" t="s">
-        <v>112</v>
-      </c>
+      <c r="A105" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B105" s="6"/>
       <c r="C105" s="1" t="s">
         <v>104</v>
       </c>
@@ -3289,7 +3238,7 @@
       <c r="M105">
         <v>0.7</v>
       </c>
-      <c r="N105">
+      <c r="N105" s="5">
         <v>0.28499999999999998</v>
       </c>
       <c r="O105">
@@ -3332,321 +3281,330 @@
         <v>97</v>
       </c>
     </row>
-    <row r="106" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="B106" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="C106" s="1" t="s">
+    <row r="106" spans="1:27" s="15" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A106" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C106" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="D106">
+      <c r="D106" s="15">
         <v>880</v>
       </c>
-      <c r="E106" t="s">
-        <v>98</v>
-      </c>
-      <c r="F106" t="s">
-        <v>98</v>
-      </c>
-      <c r="G106">
+      <c r="E106" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="F106" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="G106" s="15">
         <v>20.292000000000002</v>
       </c>
-      <c r="H106">
+      <c r="H106" s="15">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="I106">
+      <c r="I106" s="15">
         <v>42.1</v>
       </c>
-      <c r="J106">
+      <c r="J106" s="15">
         <v>-41.71</v>
       </c>
-      <c r="K106">
+      <c r="K106" s="15">
         <v>0.24</v>
       </c>
-      <c r="L106">
+      <c r="L106" s="15">
         <v>15.4</v>
       </c>
-      <c r="M106">
+      <c r="M106" s="15">
         <v>0.3</v>
       </c>
-      <c r="N106">
+      <c r="N106" s="15">
         <v>0.21299999999999999</v>
       </c>
-      <c r="O106">
+      <c r="O106" s="15">
         <v>1.6E-2</v>
       </c>
-      <c r="P106">
+      <c r="P106" s="15">
         <v>238</v>
       </c>
-      <c r="Q106">
+      <c r="Q106" s="15">
         <v>4</v>
       </c>
-      <c r="R106">
+      <c r="R106" s="15">
         <v>50715.29</v>
       </c>
-      <c r="S106">
+      <c r="S106" s="15">
         <v>0.21</v>
       </c>
-      <c r="T106">
+      <c r="T106" s="15">
         <v>4.21</v>
       </c>
-      <c r="U106">
+      <c r="U106" s="15">
         <v>0.08</v>
       </c>
-      <c r="V106" s="2">
+      <c r="V106" s="15">
         <v>7.1999999999999998E-3</v>
       </c>
-      <c r="W106" s="2">
+      <c r="W106" s="15">
         <v>4.0000000000000002E-4</v>
       </c>
-      <c r="X106">
+      <c r="X106" s="15">
         <v>0.77</v>
       </c>
-      <c r="Y106">
+      <c r="Y106" s="15">
         <v>31</v>
       </c>
-      <c r="Z106" t="s">
+      <c r="Z106" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="AA106" t="s">
+      <c r="AA106" s="15" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="107" spans="1:27" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C107" s="22" t="s">
+    <row r="107" spans="1:27" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A107" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="B107" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C107" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="D107" s="21">
+      <c r="D107" s="23">
         <v>4710</v>
       </c>
-      <c r="E107" s="21" t="s">
-        <v>98</v>
-      </c>
-      <c r="F107" s="21" t="s">
-        <v>98</v>
-      </c>
-      <c r="G107" s="21">
+      <c r="E107" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="F107" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="G107" s="23">
         <v>21.340699999999998</v>
       </c>
-      <c r="H107" s="21">
+      <c r="H107" s="23">
         <v>6.9999999999999999E-4</v>
       </c>
-      <c r="I107" s="21">
+      <c r="I107" s="23">
         <v>203.7</v>
       </c>
-      <c r="J107" s="21">
+      <c r="J107" s="23">
         <v>-45.7</v>
       </c>
-      <c r="K107" s="21">
+      <c r="K107" s="23">
         <v>0.3</v>
       </c>
-      <c r="L107" s="21">
+      <c r="L107" s="23">
         <v>16.899999999999999</v>
       </c>
-      <c r="M107" s="21">
+      <c r="M107" s="23">
         <v>1.5</v>
       </c>
-      <c r="N107" s="21">
+      <c r="N107" s="25">
         <v>0.67500000000000004</v>
       </c>
-      <c r="O107" s="21">
+      <c r="O107" s="23">
         <v>2.4E-2</v>
       </c>
-      <c r="P107" s="21">
+      <c r="P107" s="23">
         <v>340</v>
       </c>
-      <c r="Q107" s="21">
+      <c r="Q107" s="23">
         <v>3</v>
       </c>
-      <c r="R107" s="21">
+      <c r="R107" s="23">
         <v>52412.34</v>
       </c>
-      <c r="S107" s="21">
+      <c r="S107" s="23">
         <v>0.16</v>
       </c>
-      <c r="T107" s="21">
+      <c r="T107" s="23">
         <v>3.7</v>
       </c>
-      <c r="U107" s="21">
+      <c r="U107" s="23">
         <v>0.3</v>
       </c>
-      <c r="V107" s="23">
+      <c r="V107" s="26">
         <v>4.3E-3</v>
       </c>
-      <c r="W107" s="23">
+      <c r="W107" s="26">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="X107" s="21">
+      <c r="X107" s="23">
         <v>1.18</v>
       </c>
-      <c r="Y107" s="21">
+      <c r="Y107" s="23">
         <v>37</v>
       </c>
-      <c r="Z107" s="21" t="s">
+      <c r="Z107" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="AA107" s="21" t="s">
+      <c r="AA107" s="23" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="108" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C108" s="8" t="s">
+    <row r="108" spans="1:27" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A108" s="8"/>
+      <c r="C108" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D108" s="10">
+      <c r="D108" s="9">
         <v>5110</v>
       </c>
-      <c r="E108" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="F108" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="G108" s="10">
+      <c r="E108" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F108" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G108" s="9">
         <v>21.360199999999999</v>
       </c>
-      <c r="H108" s="10">
+      <c r="H108" s="9">
         <v>1.9E-3</v>
       </c>
-      <c r="I108" s="10">
+      <c r="I108" s="9">
         <v>163.19999999999999</v>
       </c>
-      <c r="J108" s="10">
+      <c r="J108" s="9">
         <v>-38</v>
       </c>
-      <c r="K108" s="10">
+      <c r="K108" s="9">
         <v>0.7</v>
       </c>
-      <c r="L108" s="10">
+      <c r="L108" s="9">
         <v>37.799999999999997</v>
       </c>
-      <c r="M108" s="10">
+      <c r="M108" s="9">
         <v>0.9</v>
       </c>
-      <c r="N108" s="10">
+      <c r="N108" s="21">
         <v>0.1</v>
       </c>
-      <c r="O108" s="10">
+      <c r="O108" s="9">
         <v>0.03</v>
       </c>
-      <c r="P108" s="10">
+      <c r="P108" s="9">
         <v>195</v>
       </c>
-      <c r="Q108" s="10">
+      <c r="Q108" s="9">
         <v>16</v>
       </c>
-      <c r="R108" s="10">
+      <c r="R108" s="9">
         <v>51197.2</v>
       </c>
-      <c r="S108" s="10">
+      <c r="S108" s="9">
         <v>0.9</v>
       </c>
-      <c r="T108" s="10">
+      <c r="T108" s="9">
         <v>11.1</v>
       </c>
-      <c r="U108" s="10">
+      <c r="U108" s="9">
         <v>0.3</v>
       </c>
-      <c r="V108" s="11">
+      <c r="V108" s="10">
         <v>0.11799999999999999</v>
       </c>
-      <c r="W108" s="11">
+      <c r="W108" s="10">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="X108" s="10">
+      <c r="X108" s="9">
         <v>3.07</v>
       </c>
-      <c r="Y108" s="10">
+      <c r="Y108" s="9">
         <v>22</v>
       </c>
-      <c r="Z108" s="10" t="s">
+      <c r="Z108" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="AA108" s="10" t="s">
+      <c r="AA108" s="9" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="109" spans="1:27" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C109" s="8" t="s">
+    <row r="109" spans="1:27" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A109" s="8"/>
+      <c r="C109" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D109" s="10">
+      <c r="D109" s="9">
         <v>736</v>
       </c>
-      <c r="E109" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="F109" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="G109" s="10">
+      <c r="E109" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F109" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G109" s="9">
         <v>24.004000000000001</v>
       </c>
-      <c r="H109" s="10">
+      <c r="H109" s="9">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="I109" s="10">
+      <c r="I109" s="9">
         <v>50.8</v>
       </c>
-      <c r="J109" s="10">
+      <c r="J109" s="9">
         <v>-50.5</v>
       </c>
-      <c r="K109" s="10">
+      <c r="K109" s="9">
         <v>0.11</v>
       </c>
-      <c r="L109" s="10">
+      <c r="L109" s="9">
         <v>7.21</v>
       </c>
-      <c r="M109" s="10">
+      <c r="M109" s="9">
         <v>0.16</v>
       </c>
-      <c r="N109" s="10">
+      <c r="N109" s="21">
         <v>0.21</v>
       </c>
-      <c r="O109" s="10">
+      <c r="O109" s="9">
         <v>1.9E-2</v>
       </c>
-      <c r="P109" s="10">
+      <c r="P109" s="9">
         <v>240</v>
       </c>
-      <c r="Q109" s="10">
+      <c r="Q109" s="9">
         <v>6</v>
       </c>
-      <c r="R109" s="10">
+      <c r="R109" s="9">
         <v>52039.8</v>
       </c>
-      <c r="S109" s="10">
+      <c r="S109" s="9">
         <v>0.4</v>
       </c>
-      <c r="T109" s="10">
+      <c r="T109" s="9">
         <v>2.33</v>
       </c>
-      <c r="U109" s="10">
+      <c r="U109" s="9">
         <v>0.05</v>
       </c>
-      <c r="V109" s="11">
+      <c r="V109" s="10">
         <v>8.7000000000000001E-4</v>
       </c>
-      <c r="W109" s="11">
+      <c r="W109" s="10">
         <v>6.0000000000000002E-5</v>
       </c>
-      <c r="X109" s="10">
+      <c r="X109" s="9">
         <v>0.42</v>
       </c>
-      <c r="Y109" s="10">
+      <c r="Y109" s="9">
         <v>17</v>
       </c>
-      <c r="Z109" s="10" t="s">
+      <c r="Z109" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="AA109" s="10" t="s">
+      <c r="AA109" s="9" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="110" spans="1:27" ht="29" x14ac:dyDescent="0.35">
-      <c r="B110" s="25" t="s">
-        <v>125</v>
-      </c>
+      <c r="A110" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="B110" s="19"/>
       <c r="C110" s="1" t="s">
         <v>104</v>
       </c>
@@ -3680,7 +3638,7 @@
       <c r="M110">
         <v>0.6</v>
       </c>
-      <c r="N110">
+      <c r="N110" s="5">
         <v>0.32</v>
       </c>
       <c r="O110">
@@ -3724,9 +3682,10 @@
       </c>
     </row>
     <row r="111" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="B111" s="24" t="s">
-        <v>112</v>
-      </c>
+      <c r="A111" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="B111" s="6"/>
       <c r="C111" s="1" t="s">
         <v>104</v>
       </c>
@@ -3760,7 +3719,7 @@
       <c r="M111">
         <v>0.3</v>
       </c>
-      <c r="N111">
+      <c r="N111" s="5">
         <v>6.9000000000000006E-2</v>
       </c>
       <c r="O111">
@@ -3804,9 +3763,10 @@
       </c>
     </row>
     <row r="112" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="B112" s="14" t="s">
-        <v>112</v>
-      </c>
+      <c r="A112" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="B112" s="18"/>
       <c r="C112" s="1" t="s">
         <v>104</v>
       </c>
@@ -3840,7 +3800,7 @@
       <c r="M112">
         <v>0.24</v>
       </c>
-      <c r="N112">
+      <c r="N112" s="5">
         <v>0.28999999999999998</v>
       </c>
       <c r="O112">
@@ -3883,84 +3843,90 @@
         <v>97</v>
       </c>
     </row>
-    <row r="113" spans="3:27" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C113" s="22" t="s">
+    <row r="113" spans="1:27" s="23" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A113" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C113" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="D113" s="21">
+      <c r="D113" s="23">
         <v>4673</v>
       </c>
-      <c r="E113" s="21" t="s">
-        <v>98</v>
-      </c>
-      <c r="F113" s="21" t="s">
-        <v>98</v>
-      </c>
-      <c r="G113" s="21">
+      <c r="E113" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="F113" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="G113" s="23">
         <v>48.27</v>
       </c>
-      <c r="H113" s="21">
+      <c r="H113" s="23">
         <v>0.06</v>
       </c>
-      <c r="I113" s="21">
+      <c r="I113" s="23">
         <v>22.4</v>
       </c>
-      <c r="J113" s="21">
+      <c r="J113" s="23">
         <v>-41.35</v>
       </c>
-      <c r="K113" s="21">
+      <c r="K113" s="23">
         <v>0.12</v>
       </c>
-      <c r="L113" s="21">
+      <c r="L113" s="23">
         <v>8.4</v>
       </c>
-      <c r="M113" s="21">
+      <c r="M113" s="23">
         <v>0.3</v>
       </c>
-      <c r="N113" s="21">
+      <c r="N113" s="25">
         <v>0.37</v>
       </c>
-      <c r="O113" s="21">
+      <c r="O113" s="23">
         <v>0.03</v>
       </c>
-      <c r="P113" s="21">
+      <c r="P113" s="23">
         <v>351</v>
       </c>
-      <c r="Q113" s="21">
+      <c r="Q113" s="23">
         <v>4</v>
       </c>
-      <c r="R113" s="21">
+      <c r="R113" s="23">
         <v>50836.6</v>
       </c>
-      <c r="S113" s="21">
+      <c r="S113" s="23">
         <v>0.6</v>
       </c>
-      <c r="T113" s="21">
+      <c r="T113" s="23">
         <v>5.18</v>
       </c>
-      <c r="U113" s="21">
+      <c r="U113" s="23">
         <v>0.19</v>
       </c>
-      <c r="V113" s="23">
+      <c r="V113" s="26">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="W113" s="23">
+      <c r="W113" s="26">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="X113" s="21">
+      <c r="X113" s="23">
         <v>0.49</v>
       </c>
-      <c r="Y113" s="21">
+      <c r="Y113" s="23">
         <v>22</v>
       </c>
-      <c r="Z113" s="21" t="s">
+      <c r="Z113" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="AA113" s="21" t="s">
+      <c r="AA113" s="23" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="114" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A114" s="11" t="s">
+        <v>111</v>
+      </c>
       <c r="C114" s="1" t="s">
         <v>104</v>
       </c>
@@ -3994,7 +3960,7 @@
       <c r="M114">
         <v>0.22</v>
       </c>
-      <c r="N114">
+      <c r="N114" s="5">
         <v>0.63300000000000001</v>
       </c>
       <c r="O114">
@@ -4037,7 +4003,10 @@
         <v>97</v>
       </c>
     </row>
-    <row r="115" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A115" s="11" t="s">
+        <v>111</v>
+      </c>
       <c r="C115" s="1" t="s">
         <v>104</v>
       </c>
@@ -4071,7 +4040,7 @@
       <c r="M115">
         <v>0.12</v>
       </c>
-      <c r="N115">
+      <c r="N115" s="5">
         <v>0.20399999999999999</v>
       </c>
       <c r="O115">
@@ -4114,7 +4083,10 @@
         <v>97</v>
       </c>
     </row>
-    <row r="116" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A116" s="11" t="s">
+        <v>111</v>
+      </c>
       <c r="C116" s="1" t="s">
         <v>104</v>
       </c>
@@ -4148,7 +4120,7 @@
       <c r="M116">
         <v>0.5</v>
       </c>
-      <c r="N116">
+      <c r="N116" s="5">
         <v>0.18</v>
       </c>
       <c r="O116">
@@ -4191,7 +4163,10 @@
         <v>97</v>
       </c>
     </row>
-    <row r="117" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A117" s="11" t="s">
+        <v>111</v>
+      </c>
       <c r="C117" s="1" t="s">
         <v>104</v>
       </c>
@@ -4225,7 +4200,7 @@
       <c r="M117">
         <v>0.3</v>
       </c>
-      <c r="N117">
+      <c r="N117" s="5">
         <v>0.31</v>
       </c>
       <c r="O117">
@@ -4268,84 +4243,87 @@
         <v>97</v>
       </c>
     </row>
-    <row r="118" spans="3:27" x14ac:dyDescent="0.2">
-      <c r="C118" s="1" t="s">
+    <row r="118" spans="1:27" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A118" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="C118" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D118">
+      <c r="D118" s="9">
         <v>5927</v>
       </c>
-      <c r="E118" t="s">
-        <v>98</v>
-      </c>
-      <c r="F118" t="s">
-        <v>98</v>
-      </c>
-      <c r="G118">
+      <c r="E118" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F118" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G118" s="9">
         <v>99.94</v>
       </c>
-      <c r="H118">
+      <c r="H118" s="9">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="I118">
+      <c r="I118" s="9">
         <v>113.5</v>
       </c>
-      <c r="J118">
+      <c r="J118" s="9">
         <v>-43.21</v>
       </c>
-      <c r="K118">
+      <c r="K118" s="9">
         <v>0.13</v>
       </c>
-      <c r="L118">
+      <c r="L118" s="9">
         <v>6.9</v>
       </c>
-      <c r="M118">
+      <c r="M118" s="9">
         <v>0.3</v>
       </c>
-      <c r="N118">
+      <c r="N118" s="21">
         <v>0.6</v>
       </c>
-      <c r="O118">
+      <c r="O118" s="9">
         <v>2.3E-2</v>
       </c>
-      <c r="P118">
+      <c r="P118" s="9">
         <v>165</v>
       </c>
-      <c r="Q118">
+      <c r="Q118" s="9">
         <v>3</v>
       </c>
-      <c r="R118">
+      <c r="R118" s="9">
         <v>48271.1</v>
       </c>
-      <c r="S118">
+      <c r="S118" s="9">
         <v>0.6</v>
       </c>
-      <c r="T118">
+      <c r="T118" s="9">
         <v>7.6</v>
       </c>
-      <c r="U118">
+      <c r="U118" s="9">
         <v>0.4</v>
       </c>
-      <c r="V118" s="2">
+      <c r="V118" s="10">
         <v>1.7799999999999999E-3</v>
       </c>
-      <c r="W118" s="2">
+      <c r="W118" s="10">
         <v>2.5000000000000001E-4</v>
       </c>
-      <c r="X118">
+      <c r="X118" s="9">
         <v>0.62</v>
       </c>
-      <c r="Y118">
+      <c r="Y118" s="9">
         <v>23</v>
       </c>
-      <c r="Z118" t="s">
+      <c r="Z118" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="AA118" t="s">
+      <c r="AA118" s="9" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="119" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:27" x14ac:dyDescent="0.2">
       <c r="C119" s="1" t="s">
         <v>104</v>
       </c>
@@ -4379,7 +4357,7 @@
       <c r="M119">
         <v>0.5</v>
       </c>
-      <c r="N119">
+      <c r="N119" s="5">
         <v>0.17100000000000001</v>
       </c>
       <c r="O119">
@@ -4422,7 +4400,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="120" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:27" x14ac:dyDescent="0.2">
       <c r="C120" s="1" t="s">
         <v>104</v>
       </c>
@@ -4456,7 +4434,7 @@
       <c r="M120">
         <v>1.1000000000000001</v>
       </c>
-      <c r="N120">
+      <c r="N120" s="5">
         <v>0.78500000000000003</v>
       </c>
       <c r="O120">
@@ -4499,7 +4477,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="121" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:27" x14ac:dyDescent="0.2">
       <c r="C121" s="1" t="s">
         <v>104</v>
       </c>
@@ -4533,7 +4511,7 @@
       <c r="M121">
         <v>0.2</v>
       </c>
-      <c r="N121">
+      <c r="N121" s="5">
         <v>0.44600000000000001</v>
       </c>
       <c r="O121">
@@ -4576,7 +4554,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="122" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:27" x14ac:dyDescent="0.2">
       <c r="C122" s="1" t="s">
         <v>104</v>
       </c>
@@ -4610,7 +4588,7 @@
       <c r="M122">
         <v>0.17</v>
       </c>
-      <c r="N122">
+      <c r="N122" s="5">
         <v>0.24</v>
       </c>
       <c r="O122">
@@ -4653,7 +4631,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="123" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:27" x14ac:dyDescent="0.2">
       <c r="C123" s="1" t="s">
         <v>104</v>
       </c>
@@ -4687,7 +4665,7 @@
       <c r="M123">
         <v>0.14000000000000001</v>
       </c>
-      <c r="N123">
+      <c r="N123" s="5">
         <v>0.129</v>
       </c>
       <c r="O123">
@@ -4730,7 +4708,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="124" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:27" x14ac:dyDescent="0.2">
       <c r="C124" s="1" t="s">
         <v>73</v>
       </c>
@@ -4764,7 +4742,7 @@
       <c r="M124">
         <v>0.3</v>
       </c>
-      <c r="N124">
+      <c r="N124" s="5">
         <v>0.16</v>
       </c>
       <c r="O124">
@@ -4807,7 +4785,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="125" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:27" x14ac:dyDescent="0.2">
       <c r="C125" s="1" t="s">
         <v>104</v>
       </c>
@@ -4841,7 +4819,7 @@
       <c r="M125">
         <v>0.4</v>
       </c>
-      <c r="N125">
+      <c r="N125" s="5">
         <v>0.37</v>
       </c>
       <c r="O125">
@@ -4884,7 +4862,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="126" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:27" x14ac:dyDescent="0.2">
       <c r="C126" s="1" t="s">
         <v>104</v>
       </c>
@@ -4918,7 +4896,7 @@
       <c r="M126">
         <v>0.6</v>
       </c>
-      <c r="N126">
+      <c r="N126" s="5">
         <v>0.71199999999999997</v>
       </c>
       <c r="O126">
@@ -4961,7 +4939,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="127" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:27" x14ac:dyDescent="0.2">
       <c r="C127" s="1" t="s">
         <v>104</v>
       </c>
@@ -4995,7 +4973,7 @@
       <c r="M127">
         <v>0.18</v>
       </c>
-      <c r="N127">
+      <c r="N127" s="5">
         <v>0.28999999999999998</v>
       </c>
       <c r="O127">
@@ -5038,7 +5016,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="128" spans="3:27" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:27" x14ac:dyDescent="0.2">
       <c r="C128" s="1" t="s">
         <v>104</v>
       </c>
@@ -5072,7 +5050,7 @@
       <c r="M128">
         <v>0.19</v>
       </c>
-      <c r="N128">
+      <c r="N128" s="5">
         <v>0.15</v>
       </c>
       <c r="O128">
@@ -5149,7 +5127,7 @@
       <c r="M129">
         <v>0.22</v>
       </c>
-      <c r="N129">
+      <c r="N129" s="5">
         <v>0.42199999999999999</v>
       </c>
       <c r="O129">
@@ -5226,7 +5204,7 @@
       <c r="M130">
         <v>0.3</v>
       </c>
-      <c r="N130">
+      <c r="N130" s="5">
         <v>0.45</v>
       </c>
       <c r="O130">
@@ -5303,7 +5281,7 @@
       <c r="M131">
         <v>0.5</v>
       </c>
-      <c r="N131">
+      <c r="N131" s="5">
         <v>0.36</v>
       </c>
       <c r="O131">
@@ -5380,7 +5358,7 @@
       <c r="M132">
         <v>0.8</v>
       </c>
-      <c r="N132">
+      <c r="N132" s="5">
         <v>0.67300000000000004</v>
       </c>
       <c r="O132">
@@ -5457,7 +5435,7 @@
       <c r="M133">
         <v>0.4</v>
       </c>
-      <c r="N133">
+      <c r="N133" s="5">
         <v>0.1</v>
       </c>
       <c r="O133">
@@ -5534,7 +5512,7 @@
       <c r="M134">
         <v>0.2</v>
       </c>
-      <c r="N134">
+      <c r="N134" s="5">
         <v>0.3</v>
       </c>
       <c r="O134">
@@ -5611,7 +5589,7 @@
       <c r="M135">
         <v>0.23</v>
       </c>
-      <c r="N135">
+      <c r="N135" s="5">
         <v>0.64100000000000001</v>
       </c>
       <c r="O135">
@@ -5688,7 +5666,7 @@
       <c r="M136">
         <v>0.4</v>
       </c>
-      <c r="N136">
+      <c r="N136" s="5">
         <v>0.44</v>
       </c>
       <c r="O136">
@@ -5765,7 +5743,7 @@
       <c r="M137">
         <v>0.19</v>
       </c>
-      <c r="N137">
+      <c r="N137" s="5">
         <v>0.49099999999999999</v>
       </c>
       <c r="O137">
@@ -5842,7 +5820,7 @@
       <c r="M138">
         <v>0.22</v>
       </c>
-      <c r="N138">
+      <c r="N138" s="5">
         <v>0.38</v>
       </c>
       <c r="O138">
@@ -5919,7 +5897,7 @@
       <c r="M139">
         <v>0.09</v>
       </c>
-      <c r="N139">
+      <c r="N139" s="5">
         <v>0.26900000000000002</v>
       </c>
       <c r="O139">
@@ -5996,7 +5974,7 @@
       <c r="M140">
         <v>0.3</v>
       </c>
-      <c r="N140">
+      <c r="N140" s="5">
         <v>0.2</v>
       </c>
       <c r="O140">
@@ -6073,7 +6051,7 @@
       <c r="M141">
         <v>0.17</v>
       </c>
-      <c r="N141">
+      <c r="N141" s="5">
         <v>0.21</v>
       </c>
       <c r="O141">
@@ -6150,7 +6128,7 @@
       <c r="M142">
         <v>0.13</v>
       </c>
-      <c r="N142">
+      <c r="N142" s="5">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="O142">
@@ -6227,7 +6205,7 @@
       <c r="M143">
         <v>0.13</v>
       </c>
-      <c r="N143">
+      <c r="N143" s="5">
         <v>0.22</v>
       </c>
       <c r="O143">
@@ -6304,7 +6282,7 @@
       <c r="M144">
         <v>0.17</v>
       </c>
-      <c r="N144">
+      <c r="N144" s="5">
         <v>0.34</v>
       </c>
       <c r="O144">
@@ -6381,7 +6359,7 @@
       <c r="M145">
         <v>0.16</v>
       </c>
-      <c r="N145">
+      <c r="N145" s="5">
         <v>0.14000000000000001</v>
       </c>
       <c r="O145">
@@ -6458,7 +6436,7 @@
       <c r="M146">
         <v>1</v>
       </c>
-      <c r="N146">
+      <c r="N146" s="5">
         <v>0.74</v>
       </c>
       <c r="O146">
@@ -6535,7 +6513,7 @@
       <c r="M147">
         <v>0.4</v>
       </c>
-      <c r="N147">
+      <c r="N147" s="5">
         <v>0.5</v>
       </c>
       <c r="O147">
@@ -6612,7 +6590,7 @@
       <c r="M148">
         <v>0.09</v>
       </c>
-      <c r="N148">
+      <c r="N148" s="5">
         <v>9.5000000000000001E-2</v>
       </c>
       <c r="O148">
@@ -6689,7 +6667,7 @@
       <c r="M149">
         <v>0.3</v>
       </c>
-      <c r="N149">
+      <c r="N149" s="5">
         <v>0.312</v>
       </c>
       <c r="O149">
@@ -6766,7 +6744,7 @@
       <c r="M150">
         <v>0.4</v>
       </c>
-      <c r="N150">
+      <c r="N150" s="5">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="O150">
@@ -6843,7 +6821,7 @@
       <c r="M151">
         <v>0.4</v>
       </c>
-      <c r="N151">
+      <c r="N151" s="5">
         <v>0.09</v>
       </c>
       <c r="O151">
@@ -6920,7 +6898,7 @@
       <c r="M152">
         <v>0.13</v>
       </c>
-      <c r="N152">
+      <c r="N152" s="5">
         <v>0.14000000000000001</v>
       </c>
       <c r="O152">
@@ -6997,7 +6975,7 @@
       <c r="M153">
         <v>1.7</v>
       </c>
-      <c r="N153">
+      <c r="N153" s="5">
         <v>0.7</v>
       </c>
       <c r="O153">
@@ -7074,7 +7052,7 @@
       <c r="M154">
         <v>0.16</v>
       </c>
-      <c r="N154">
+      <c r="N154" s="5">
         <v>0.21</v>
       </c>
       <c r="O154">
@@ -7151,7 +7129,7 @@
       <c r="M155">
         <v>0.16</v>
       </c>
-      <c r="N155">
+      <c r="N155" s="5">
         <v>0.09</v>
       </c>
       <c r="O155">
@@ -7228,7 +7206,7 @@
       <c r="M156">
         <v>0.3</v>
       </c>
-      <c r="N156">
+      <c r="N156" s="5">
         <v>0.25</v>
       </c>
       <c r="O156">
@@ -7305,7 +7283,7 @@
       <c r="M157">
         <v>0.3</v>
       </c>
-      <c r="N157">
+      <c r="N157" s="5">
         <v>0.55100000000000005</v>
       </c>
       <c r="O157">
@@ -7382,7 +7360,7 @@
       <c r="M158">
         <v>0.9</v>
       </c>
-      <c r="N158">
+      <c r="N158" s="5">
         <v>0.37</v>
       </c>
       <c r="O158">
@@ -7459,7 +7437,7 @@
       <c r="M159">
         <v>0.5</v>
       </c>
-      <c r="N159">
+      <c r="N159" s="5">
         <v>0.63</v>
       </c>
       <c r="O159">
@@ -7536,7 +7514,7 @@
       <c r="M160">
         <v>0.1</v>
       </c>
-      <c r="N160">
+      <c r="N160" s="5">
         <v>0.28599999999999998</v>
       </c>
       <c r="O160">
@@ -7613,7 +7591,7 @@
       <c r="M161">
         <v>0.7</v>
       </c>
-      <c r="N161">
+      <c r="N161" s="5">
         <v>0.45</v>
       </c>
       <c r="O161">
@@ -7690,7 +7668,7 @@
       <c r="M162">
         <v>0.8</v>
       </c>
-      <c r="N162">
+      <c r="N162" s="5">
         <v>0.77</v>
       </c>
       <c r="O162">
@@ -7767,7 +7745,7 @@
       <c r="M163">
         <v>0.23</v>
       </c>
-      <c r="N163">
+      <c r="N163" s="5">
         <v>0.54</v>
       </c>
       <c r="O163">
@@ -7844,7 +7822,7 @@
       <c r="M164">
         <v>0.4</v>
       </c>
-      <c r="N164">
+      <c r="N164" s="5">
         <v>0.21</v>
       </c>
       <c r="O164">
@@ -7921,7 +7899,7 @@
       <c r="M165">
         <v>0.3</v>
       </c>
-      <c r="N165">
+      <c r="N165" s="5">
         <v>0.32</v>
       </c>
       <c r="O165">
@@ -7998,7 +7976,7 @@
       <c r="M166">
         <v>0.13</v>
       </c>
-      <c r="N166">
+      <c r="N166" s="5">
         <v>0.15</v>
       </c>
       <c r="O166">
@@ -8075,7 +8053,7 @@
       <c r="M167">
         <v>0.12</v>
       </c>
-      <c r="N167">
+      <c r="N167" s="5">
         <v>0.31</v>
       </c>
       <c r="O167">
@@ -8152,7 +8130,7 @@
       <c r="M168">
         <v>0.4</v>
       </c>
-      <c r="N168">
+      <c r="N168" s="5">
         <v>0.36</v>
       </c>
       <c r="O168">
@@ -8229,7 +8207,7 @@
       <c r="M169">
         <v>0.24</v>
       </c>
-      <c r="N169">
+      <c r="N169" s="5">
         <v>0.38</v>
       </c>
       <c r="O169">
@@ -8306,7 +8284,7 @@
       <c r="M170">
         <v>0.3</v>
       </c>
-      <c r="N170">
+      <c r="N170" s="5">
         <v>0.15</v>
       </c>
       <c r="O170">
@@ -8383,7 +8361,7 @@
       <c r="M171">
         <v>1.6</v>
       </c>
-      <c r="N171">
+      <c r="N171" s="5">
         <v>0.86</v>
       </c>
       <c r="O171">
@@ -8460,7 +8438,7 @@
       <c r="M172">
         <v>0.09</v>
       </c>
-      <c r="N172">
+      <c r="N172" s="5">
         <v>0.51100000000000001</v>
       </c>
       <c r="O172">

</xml_diff>